<commit_message>
lsaeb enum signal added
</commit_message>
<xml_diff>
--- a/config/signal_map.xlsx
+++ b/config/signal_map.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B26F7940-EF16-3443-8E4A-E9ACD37E1201}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF3813F1-2E9E-1E42-A15C-8FBB6DD8542F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="20360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="57">
   <si>
     <t>payload/long_ctrl_accel_request</t>
   </si>
@@ -199,6 +199,12 @@
   </si>
   <si>
     <t>fcw_state_info/time_to_collision</t>
+  </si>
+  <si>
+    <t>active_safety_status/notices/CPM/braking_event_status</t>
+  </si>
+  <si>
+    <t>cpmEventType</t>
   </si>
 </sst>
 </file>
@@ -905,9 +911,18 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="5"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="5"/>
+      <c r="A23" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D23" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="5"/>

</xml_diff>

<commit_message>
start to integrate lka feature
</commit_message>
<xml_diff>
--- a/config/signal_map.xlsx
+++ b/config/signal_map.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01BB2A46-3CD9-3B4F-9FD9-C07B6A6C4F79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8C0F448-4C35-FF4F-9114-C4FF63DA49E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="20360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="71">
   <si>
     <t>payload/long_ctrl_accel_request</t>
   </si>
@@ -220,6 +220,33 @@
   </si>
   <si>
     <t>cpmLatDist</t>
+  </si>
+  <si>
+    <t>active_safety_status/notices/LKA/intervention_status</t>
+  </si>
+  <si>
+    <t>lkaInterventionStatus</t>
+  </si>
+  <si>
+    <t>LaneSupportSystemDebug</t>
+  </si>
+  <si>
+    <t>dtle_actuation_threshold</t>
+  </si>
+  <si>
+    <t>dtleTarget</t>
+  </si>
+  <si>
+    <t>current_DTLE</t>
+  </si>
+  <si>
+    <t>dtle</t>
+  </si>
+  <si>
+    <t>steering_wheel_torque</t>
+  </si>
+  <si>
+    <t>steerWheelTorque</t>
   </si>
 </sst>
 </file>
@@ -968,24 +995,60 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="5"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="5"/>
+      <c r="A26" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="D26" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="5"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="5"/>
+      <c r="A27" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D27" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="5"/>
-      <c r="B28" s="4"/>
-      <c r="C28" s="5"/>
+      <c r="A28" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D28" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="5"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="5"/>
+      <c r="A29" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D29" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="5"/>

</xml_diff>

<commit_message>
move base class out of as_long
</commit_message>
<xml_diff>
--- a/config/signal_map.xlsx
+++ b/config/signal_map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF8BE73E-E2FF-2C4F-A8F2-F309D7643BBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{459F6701-3570-0C49-A5D2-05ECDF860AA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="20360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="45120" yWindow="5480" windowWidth="34200" windowHeight="13760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vbRcSignals" sheetId="1" r:id="rId1"/>

</xml_diff>